<commit_message>
Revisi semua deliverables keuangan — data aktual Juni 2026
Update 6 file laporan keuangan berdasarkan tagihan aktual BCA (3 Jun 2026)
dan DBS (25 Mei 2026), klarifikasi Microsoft 365 tahunan, dan identifikasi
4 AUTOPAY BCA sebagai MyRepublic Internet 4 lokasi.

Koreksi utama:
- BCA saldo: Rp 10,3 juta → Rp 25,3 juta (aktual tagihan)
- DBS saldo: Rp 1,08 juta → Rp 9.057 (hampir lunas, JT 10 Jun bukan 12)
- Total hutang aktif: Rp 107,7 juta → Rp 120,1 juta
- Target bebas hutang: April 2027 (BCA lunas Apr, bukan Mar)
- Microsoft 365: Rp 31.999/bln → Rp 1.699.999/TAHUN (perpanjang Mei 2027)
- Netflix kartu: BNI Lotte 2256 → BCA Visa 6319
- 4 AUTOPAY: "tidak teridentifikasi" → MyRepublic Internet 4 lokasi
- HBOMax: CIMB 5022 sudah DITUTUP — perlu cek kartu baru
- CIMB Visa 5022 & BNI Visa 8379: DITUTUP Juni 2026

https://claude.ai/code/session_01QvEtyuXJyvv9G7A9kGiNJZ
</commit_message>
<xml_diff>
--- a/financial-reports/Suwandhy_FinancialPlan_2026-2027.xlsx
+++ b/financial-reports/Suwandhy_FinancialPlan_2026-2027.xlsx
@@ -231,7 +231,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -253,11 +253,55 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -641,6 +685,8 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1030,11 +1076,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generate: 28 Mei 2026  |  Data: Siklus Tagihan Mei 2026  |  Budget Juni 2026: Rp 12.500.000</t>
+          <t>Diperbarui: 7 Juni 2026  |  Data: Tagihan Aktual Jun 2026  |  Budget Juni 2026: Rp 12.500.000</t>
         </is>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -1202,12 +1254,12 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Bayar</t>
+          <t>🔴 OVERDUE</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>SEGERA</t>
         </is>
       </c>
     </row>
@@ -1331,12 +1383,12 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Bayar</t>
+          <t>DITUTUP</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>✅ LUNAS</t>
         </is>
       </c>
     </row>
@@ -1460,12 +1512,12 @@
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>Bayar</t>
+          <t>DITUTUP</t>
         </is>
       </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
-          <t>Kecil</t>
+          <t>✅ LUNAS</t>
         </is>
       </c>
     </row>
@@ -1578,23 +1630,23 @@
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>12-Mei-26*</t>
+          <t>10-Jun-26</t>
         </is>
       </c>
       <c r="F22" s="16" t="n">
-        <v>1086557</v>
+        <v>9057</v>
       </c>
       <c r="G22" s="17" t="n">
-        <v>54327</v>
+        <v>0</v>
       </c>
       <c r="H22" s="20" t="inlineStr">
         <is>
-          <t>Tgl Mei</t>
+          <t>LUNAS Jun</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>KRITIS</t>
         </is>
       </c>
     </row>
@@ -1616,28 +1668,28 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>03-Mei-26</t>
+          <t>03-Jun-26</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>19-Mei-26*</t>
+          <t>19-Jun-26</t>
         </is>
       </c>
       <c r="F23" s="8" t="n">
-        <v>10392031</v>
+        <v>25345522</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>3367269</v>
+        <v>3882015</v>
       </c>
       <c r="H23" s="20" t="inlineStr">
         <is>
-          <t>Tgl Mei</t>
+          <t>Bayar 19Jun</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>TINGGI</t>
         </is>
       </c>
     </row>
@@ -1647,12 +1699,12 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B24" s="22" t="n"/>
-      <c r="C24" s="22" t="n"/>
-      <c r="D24" s="22" t="n"/>
-      <c r="E24" s="22" t="n"/>
+      <c r="B24" s="129" t="n"/>
+      <c r="C24" s="129" t="n"/>
+      <c r="D24" s="129" t="n"/>
+      <c r="E24" s="130" t="n"/>
       <c r="F24" s="23" t="n">
-        <v>107717747</v>
+        <v>120103899</v>
       </c>
       <c r="G24" s="23" t="n">
         <v>9944600</v>
@@ -1705,7 +1757,7 @@
       </c>
       <c r="B3" s="126" t="inlineStr">
         <is>
-          <t>Mei 2026 (transaksi Apr-Mei 2026). DBS &amp; BCA = Siklus April 2026.</t>
+          <t>Juni 2026 (tagihan aktual BCA 3 Jun + DBS 25 Mei). Total saldo terverifikasi Rp 120.103.899</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1781,7 @@
       </c>
       <c r="B5" s="126" t="inlineStr">
         <is>
-          <t>Email diterima 28 Mei 2026 via Gmail, BELUM ada di Drive</t>
+          <t>Tagihan aktual diterima 3 Juni 2026 — saldo Rp 25.345.522 (lebih Rp 15,3 juta dari estimasi awal)</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1793,7 @@
       </c>
       <c r="B6" s="128" t="inlineStr">
         <is>
-          <t>Tidak ditemukan di Gmail/Drive — hanya April 2026 tersedia</t>
+          <t>Tagihan aktual 25 Mei 2026 — saldo Rp 9.057 (hampir lunas!); JT 10 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1865,7 @@
       </c>
       <c r="B15" s="126" t="inlineStr">
         <is>
-          <t>Mandiri 3517 | Mega 6566 | CIMB Accor 0407 | CIMB Syariah 6174</t>
+          <t>Mandiri 3517 | Mega 6566 | CIMB Accor 0407 | CIMB Syariah 6174 | CIMB Visa 5022 (DITUTUP) | BNI Visa 8379 (DITUTUP)</t>
         </is>
       </c>
     </row>
@@ -1966,7 +2018,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="24" t="inlineStr">
         <is>
-          <t>SALDO &amp; LIMIT KARTU KREDIT — Mei 2026</t>
+          <t>SALDO &amp; LIMIT KARTU KREDIT — Juni 2026 (Data Aktual)</t>
         </is>
       </c>
     </row>
@@ -2249,10 +2301,10 @@
         <v>87774270</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>1478218</v>
+        <v>0</v>
       </c>
       <c r="G8" s="35" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="H8" s="41" t="inlineStr"/>
       <c r="I8" s="36" t="inlineStr">
@@ -2262,7 +2314,7 @@
       </c>
       <c r="J8" s="29" t="inlineStr">
         <is>
-          <t>Lancar</t>
+          <t>DITUTUP Jun 2026</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2421,7 @@
         <v>32488300</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>11621</v>
+        <v>0</v>
       </c>
       <c r="G11" s="37" t="n">
         <v>0</v>
@@ -2382,7 +2434,7 @@
       </c>
       <c r="J11" s="29" t="inlineStr">
         <is>
-          <t>Lancar</t>
+          <t>DITUTUP Jun 2026</t>
         </is>
       </c>
     </row>
@@ -2486,13 +2538,13 @@
         <v>12500000</v>
       </c>
       <c r="E14" s="33" t="n">
-        <v>11413443</v>
+        <v>12490943</v>
       </c>
       <c r="F14" s="34" t="n">
-        <v>1086557</v>
+        <v>9057</v>
       </c>
       <c r="G14" s="35" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.001</v>
       </c>
       <c r="H14" s="41" t="inlineStr"/>
       <c r="I14" s="36" t="inlineStr">
@@ -2502,7 +2554,7 @@
       </c>
       <c r="J14" s="29" t="inlineStr">
         <is>
-          <t>Lancar</t>
+          <t>LUNAS Jun 2026</t>
         </is>
       </c>
     </row>
@@ -2526,13 +2578,13 @@
         <v>94000000</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>77270940</v>
+        <v>68654478</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>10392031</v>
+        <v>25345522</v>
       </c>
       <c r="G15" s="37" t="n">
-        <v>0.111</v>
+        <v>0.27</v>
       </c>
       <c r="H15" s="9" t="n">
         <v>6337029</v>
@@ -2554,8 +2606,8 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B16" s="22" t="n"/>
-      <c r="C16" s="22" t="n"/>
+      <c r="B16" s="129" t="n"/>
+      <c r="C16" s="130" t="n"/>
       <c r="D16" s="43" t="n">
         <v>788000000</v>
       </c>
@@ -2563,7 +2615,7 @@
         <v>628681376</v>
       </c>
       <c r="F16" s="44" t="n">
-        <v>107717747</v>
+        <v>120103899</v>
       </c>
       <c r="G16" s="22" t="n"/>
       <c r="H16" s="43" t="n">
@@ -2604,17 +2656,18 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="45" t="inlineStr">
         <is>
-          <t>CHECKLIST PEMBAYARAN JUNI 2026 — Budget Rp 12.500.000</t>
+          <t>CHECKLIST PEMBAYARAN JUNI 2026 — Budget Rp 12.500.000 | Status: 7 Juni 2026</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="46" t="inlineStr">
         <is>
-          <t>SUDAH DIBAYAR: Mandiri 3517 | Mega 6566 | CIMB Accor 0407 | CIMB Syariah 6174</t>
-        </is>
-      </c>
-    </row>
+          <t>SUDAH DIBAYAR: Mandiri 3517 ✅ | Mega 6566 ✅ | CIMB Accor 0407 ✅ | CIMB Syariah 6174 ✅ | CIMB Visa 5022 ✅ DITUTUP | BNI Visa 8379 ✅ DITUTUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -2923,7 +2976,7 @@
       </c>
       <c r="G11" s="57" t="inlineStr">
         <is>
-          <t>BELUM</t>
+          <t>V LUNAS min</t>
         </is>
       </c>
       <c r="H11" s="51" t="n">
@@ -3003,7 +3056,7 @@
       </c>
       <c r="G13" s="57" t="inlineStr">
         <is>
-          <t>BELUM</t>
+          <t>V LUNAS — DITUTUP</t>
         </is>
       </c>
       <c r="H13" s="51" t="n">
@@ -3042,7 +3095,7 @@
       </c>
       <c r="G14" s="57" t="inlineStr">
         <is>
-          <t>BELUM</t>
+          <t>V LUNAS — DITUTUP</t>
         </is>
       </c>
       <c r="H14" s="51" t="n">
@@ -3109,24 +3162,18 @@
           <t>~19-Jun-26</t>
         </is>
       </c>
-      <c r="D16" s="62" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E16" s="62" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F16" s="63" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
+      <c r="D16" s="62" t="n">
+        <v>25345522</v>
+      </c>
+      <c r="E16" s="62" t="n">
+        <v>3882015</v>
+      </c>
+      <c r="F16" s="63" t="n">
+        <v>3882015</v>
       </c>
       <c r="G16" s="42" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Bayar 19Jun</t>
         </is>
       </c>
       <c r="H16" s="51" t="n">
@@ -3152,15 +3199,15 @@
     <row r="18">
       <c r="A18" s="21" t="inlineStr">
         <is>
-          <t>TOTAL REKOMEN BAYAR JUNI (tanpa BCA)</t>
-        </is>
-      </c>
-      <c r="B18" s="22" t="n"/>
-      <c r="C18" s="22" t="n"/>
+          <t>TOTAL REKOMEN BAYAR JUNI (incl. BCA minimum)</t>
+        </is>
+      </c>
+      <c r="B18" s="129" t="n"/>
+      <c r="C18" s="130" t="n"/>
       <c r="D18" s="22" t="n"/>
       <c r="E18" s="22" t="n"/>
       <c r="F18" s="23" t="n">
-        <v>8994627</v>
+        <v>15997911</v>
       </c>
       <c r="G18" s="22" t="n"/>
       <c r="H18" s="22" t="n"/>
@@ -3182,7 +3229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3201,7 +3248,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="65" t="inlineStr">
         <is>
-          <t>JADWAL PEMBAYARAN BULANAN — Jun 2026 s/d Mar 2027 (PROYEKSI)</t>
+          <t>JADWAL PEMBAYARAN BULANAN — Jun 2026 s/d Apr 2027 (REVISI 7 Juni 2026)</t>
         </is>
       </c>
     </row>
@@ -3345,32 +3392,50 @@
       <c r="B5" s="66" t="n">
         <v>2271312</v>
       </c>
-      <c r="C5" s="66" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D5" s="66" t="n">
-        <v>150000</v>
-      </c>
-      <c r="E5" s="66" t="n">
-        <v>150000</v>
-      </c>
-      <c r="F5" s="66" t="n">
-        <v>150000</v>
-      </c>
-      <c r="G5" s="66" t="n">
-        <v>150000</v>
-      </c>
-      <c r="H5" s="66" t="n">
-        <v>150000</v>
-      </c>
-      <c r="I5" s="66" t="n">
-        <v>150000</v>
-      </c>
-      <c r="J5" s="66" t="n">
-        <v>150000</v>
-      </c>
-      <c r="K5" s="66" t="n">
-        <v>150000</v>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -3460,19 +3525,27 @@
         </is>
       </c>
       <c r="B8" s="67" t="n">
-        <v>73911</v>
-      </c>
-      <c r="C8" s="67" t="n">
-        <v>73911</v>
-      </c>
-      <c r="D8" s="67" t="n">
-        <v>73911</v>
-      </c>
-      <c r="E8" s="67" t="n">
-        <v>73911</v>
-      </c>
-      <c r="F8" s="67" t="n">
-        <v>600000</v>
+        <v>1478218</v>
+      </c>
+      <c r="C8" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G8" s="69" t="inlineStr">
         <is>
@@ -3720,31 +3793,47 @@
         </is>
       </c>
       <c r="B14" s="67" t="n">
-        <v>54327</v>
-      </c>
-      <c r="C14" s="67" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D14" s="67" t="n">
-        <v>100000</v>
-      </c>
-      <c r="E14" s="67" t="n">
-        <v>100000</v>
-      </c>
-      <c r="F14" s="67" t="n">
-        <v>100000</v>
-      </c>
-      <c r="G14" s="67" t="n">
-        <v>100000</v>
-      </c>
-      <c r="H14" s="67" t="n">
-        <v>100000</v>
-      </c>
-      <c r="I14" s="67" t="n">
-        <v>100000</v>
-      </c>
-      <c r="J14" s="67" t="n">
-        <v>100000</v>
+        <v>9057</v>
+      </c>
+      <c r="C14" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" s="67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K14" s="69" t="inlineStr">
         <is>
@@ -3759,34 +3848,34 @@
         </is>
       </c>
       <c r="B15" s="66" t="n">
-        <v>3367269</v>
+        <v>3882015</v>
       </c>
       <c r="C15" s="66" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="D15" s="66" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="E15" s="66" t="n">
         <v>3000000</v>
       </c>
-      <c r="D15" s="66" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="E15" s="66" t="n">
-        <v>2500000</v>
-      </c>
       <c r="F15" s="66" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="G15" s="66" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="H15" s="66" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="I15" s="66" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="J15" s="66" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="K15" s="66" t="n">
         <v>2000000</v>
-      </c>
-      <c r="G15" s="66" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="H15" s="66" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="I15" s="66" t="n">
-        <v>500000</v>
-      </c>
-      <c r="J15" s="66" t="n">
-        <v>500000</v>
-      </c>
-      <c r="K15" s="66" t="n">
-        <v>500000</v>
       </c>
     </row>
     <row r="16">
@@ -4874,8 +4963,8 @@
           <t>TOTAL SISA CICILAN</t>
         </is>
       </c>
-      <c r="B23" s="22" t="n"/>
-      <c r="C23" s="22" t="n"/>
+      <c r="B23" s="129" t="n"/>
+      <c r="C23" s="130" t="n"/>
       <c r="D23" s="83" t="n">
         <v>15243078</v>
       </c>
@@ -4918,7 +5007,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="24" t="inlineStr">
         <is>
-          <t>TRACKER LANGGANAN &amp; PROTEKSI — Mei 2026</t>
+          <t>TRACKER LANGGANAN &amp; PROTEKSI — Update 7 Juni 2026</t>
         </is>
       </c>
     </row>
@@ -4972,7 +5061,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>BCA 6319 + BNI Lotte 2256</t>
+          <t>BCA Visa 6319</t>
         </is>
       </c>
       <c r="D3" s="9" t="n">
@@ -4985,7 +5074,7 @@
       </c>
       <c r="F3" s="85" t="inlineStr">
         <is>
-          <t>MUNGKIN DUPLIKAT (2x tagihan)!</t>
+          <t>Aktif BCA 6319</t>
         </is>
       </c>
       <c r="G3" s="86" t="n">
@@ -5269,7 +5358,7 @@
     <row r="12">
       <c r="A12" s="30" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Microsoft 365 Family (TAHUNAN)</t>
         </is>
       </c>
       <c r="B12" s="31" t="inlineStr">
@@ -5283,7 +5372,7 @@
         </is>
       </c>
       <c r="D12" s="33" t="n">
-        <v>31999</v>
+        <v>141667</v>
       </c>
       <c r="E12" s="29" t="inlineStr">
         <is>
@@ -5292,7 +5381,7 @@
       </c>
       <c r="F12" s="87" t="inlineStr">
         <is>
-          <t>Office suite terjangkau</t>
+          <t>TAHUNAN Rp1.699.999 — perpanjang Mei 2027</t>
         </is>
       </c>
       <c r="G12" s="88" t="inlineStr">
@@ -5314,7 +5403,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>CIMB Visa 5022</t>
+          <t>CIMB Visa 5022 (DITUTUP — cek kartu baru)</t>
         </is>
       </c>
       <c r="D13" s="90" t="n">
@@ -5327,7 +5416,7 @@
       </c>
       <c r="F13" s="85" t="inlineStr">
         <is>
-          <t>Mahal - evaluasi</t>
+          <t>CIMB 5022 DITUTUP — batalkan atau pindahkan kartu</t>
         </is>
       </c>
       <c r="G13" s="86" t="n">
@@ -5817,8 +5906,8 @@
           <t>KEEP - Total/bln</t>
         </is>
       </c>
-      <c r="B29" s="22" t="n"/>
-      <c r="C29" s="22" t="n"/>
+      <c r="B29" s="129" t="n"/>
+      <c r="C29" s="130" t="n"/>
       <c r="D29" s="51" t="n">
         <v>519289</v>
       </c>
@@ -5834,8 +5923,8 @@
           <t>REVIEW - Total/bln</t>
         </is>
       </c>
-      <c r="B30" s="22" t="n"/>
-      <c r="C30" s="22" t="n"/>
+      <c r="B30" s="129" t="n"/>
+      <c r="C30" s="130" t="n"/>
       <c r="D30" s="39" t="n">
         <v>2280528</v>
       </c>
@@ -5851,8 +5940,8 @@
           <t>CANCEL - Total hemat/bln</t>
         </is>
       </c>
-      <c r="B31" s="22" t="n"/>
-      <c r="C31" s="22" t="n"/>
+      <c r="B31" s="129" t="n"/>
+      <c r="C31" s="130" t="n"/>
       <c r="D31" s="27" t="n">
         <v>4225529</v>
       </c>
@@ -5868,8 +5957,8 @@
           <t>TOTAL POTENSI HEMAT/BLN</t>
         </is>
       </c>
-      <c r="B32" s="22" t="n"/>
-      <c r="C32" s="22" t="n"/>
+      <c r="B32" s="129" t="n"/>
+      <c r="C32" s="130" t="n"/>
       <c r="D32" s="95" t="n">
         <v>7025346</v>
       </c>
@@ -5912,7 +6001,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="65" t="inlineStr">
         <is>
-          <t>TRACKER UTILITAS — Autopay BCA + Faktur Langsung</t>
+          <t>TRACKER UTILITAS — Autopay BCA + Faktur Langsung | Update 7 Juni 2026</t>
         </is>
       </c>
     </row>
@@ -6236,7 +6325,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Autopay TBD</t>
+          <t>MyRepublic Internet Lokasi 1</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -6254,24 +6343,24 @@
       </c>
       <c r="E11" s="85" t="inlineStr">
         <is>
-          <t>IDENTIFIKASI!</t>
+          <t>MyRepublic internet — MyRepublic Internet Lokasi 1</t>
         </is>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Aktif</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Evaluasi</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>Autopay TBD</t>
+          <t>MyRepublic Internet Lokasi 2</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
@@ -6289,24 +6378,24 @@
       </c>
       <c r="E12" s="97" t="inlineStr">
         <is>
-          <t>IDENTIFIKASI!</t>
+          <t>MyRepublic internet — MyRepublic Internet Lokasi 2</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Aktif</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Evaluasi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Autopay TBD</t>
+          <t>MyRepublic Internet Lokasi 3</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -6324,24 +6413,24 @@
       </c>
       <c r="E13" s="85" t="inlineStr">
         <is>
-          <t>IDENTIFIKASI!</t>
+          <t>MyRepublic internet — MyRepublic Internet Lokasi 3</t>
         </is>
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Aktif</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Evaluasi</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Autopay TBD</t>
+          <t>MyRepublic Internet Lokasi 4</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
@@ -6359,17 +6448,17 @@
       </c>
       <c r="E14" s="97" t="inlineStr">
         <is>
-          <t>IDENTIFIKASI!</t>
+          <t>MyRepublic internet — MyRepublic Internet Lokasi 4</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Aktif</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Evaluasi</t>
         </is>
       </c>
     </row>
@@ -6379,8 +6468,8 @@
           <t>TOTAL UTILITAS/BLN</t>
         </is>
       </c>
-      <c r="B15" s="22" t="n"/>
-      <c r="C15" s="22" t="n"/>
+      <c r="B15" s="129" t="n"/>
+      <c r="C15" s="130" t="n"/>
       <c r="D15" s="23" t="n">
         <v>4985997</v>
       </c>
@@ -7000,7 +7089,7 @@
           <t>TOTAL BIAYA TAHUNAN</t>
         </is>
       </c>
-      <c r="B18" s="22" t="n"/>
+      <c r="B18" s="130" t="n"/>
       <c r="C18" s="44" t="n">
         <v>900000</v>
       </c>
@@ -7015,7 +7104,7 @@
           <t>TOTAL BIAYA BULANAN (tanpa cicilan)</t>
         </is>
       </c>
-      <c r="B19" s="22" t="n"/>
+      <c r="B19" s="130" t="n"/>
       <c r="C19" s="22" t="n"/>
       <c r="D19" s="44" t="n">
         <v>535000</v>
@@ -7081,7 +7170,8 @@
 • BATALKAN: semua Credit Shield/Protector (hemat ~Rp755K/bln)
 • BATALKAN: BSI Monthly Fee -&gt; pertimbangkan TUTUP kartu
 • BATALKAN: Google Transkriptor Rp2.2jt/bln!
-• IDENTIFIKASI: 4 Autopay BCA yang tidak dikenal</t>
+• TERIDENTIFIKASI: 4 Autopay BCA = MyRepublic Internet 4 lokasi (Rp 2.245.000/bln)
+• Evaluasi: tutup lokasi MyRepublic yang tidak aktif</t>
         </is>
       </c>
     </row>
@@ -7188,8 +7278,8 @@
           <t>POTENSI PENGHEMATAN JIKA REKOMENDASI DILAKSANAKAN</t>
         </is>
       </c>
-      <c r="B10" s="22" t="n"/>
-      <c r="C10" s="22" t="n"/>
+      <c r="B10" s="129" t="n"/>
+      <c r="C10" s="130" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="118" t="inlineStr">
@@ -7197,7 +7287,7 @@
           <t>Batalkan semua Credit Shield/Protector</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n"/>
+      <c r="B11" s="130" t="n"/>
       <c r="C11" s="119" t="inlineStr">
         <is>
           <t>~Rp 755,000/bln</t>
@@ -7210,7 +7300,7 @@
           <t>Batalkan BSI Monthly Fee (tutup kartu)</t>
         </is>
       </c>
-      <c r="B12" s="22" t="n"/>
+      <c r="B12" s="130" t="n"/>
       <c r="C12" s="121" t="inlineStr">
         <is>
           <t>~Rp 437,500/bln</t>
@@ -7223,7 +7313,7 @@
           <t>Batalkan Google Transkriptor</t>
         </is>
       </c>
-      <c r="B13" s="22" t="n"/>
+      <c r="B13" s="130" t="n"/>
       <c r="C13" s="119" t="inlineStr">
         <is>
           <t>~Rp 2,208,900/bln</t>
@@ -7236,7 +7326,7 @@
           <t>Batalkan Paddle.NET (setelah identifikasi)</t>
         </is>
       </c>
-      <c r="B14" s="22" t="n"/>
+      <c r="B14" s="130" t="n"/>
       <c r="C14" s="121" t="inlineStr">
         <is>
           <t>~Rp 780,199/bln</t>
@@ -7249,7 +7339,7 @@
           <t>Review HBOMax</t>
         </is>
       </c>
-      <c r="B15" s="22" t="n"/>
+      <c r="B15" s="130" t="n"/>
       <c r="C15" s="119" t="inlineStr">
         <is>
           <t>~Rp 549,000/bln</t>
@@ -7262,10 +7352,10 @@
           <t>TOTAL POTENSI HEMAT/BLN</t>
         </is>
       </c>
-      <c r="B16" s="22" t="n"/>
+      <c r="B16" s="130" t="n"/>
       <c r="C16" s="123" t="inlineStr">
         <is>
-          <t>~Rp 4,730,599/bln</t>
+          <t>~Rp 5.790.599/bln</t>
         </is>
       </c>
     </row>
@@ -7275,10 +7365,10 @@
           <t>TOTAL POTENSI HEMAT/TAHUN</t>
         </is>
       </c>
-      <c r="B17" s="22" t="n"/>
+      <c r="B17" s="130" t="n"/>
       <c r="C17" s="123" t="inlineStr">
         <is>
-          <t>~Rp 56,767,188/thn</t>
+          <t>~Rp 69.491.384/thn</t>
         </is>
       </c>
     </row>

</xml_diff>